<commit_message>
Add data processing scripts and initial data files
- Implemented data reading from JSON and added sample DataFrame creation.
- Created multiple scripts for data manipulation and analysis.
- Added initial data files: students.json and students.csv.
- Included descriptive statistics and filtering examples in new scripts.
</commit_message>
<xml_diff>
--- a/students.xlsx
+++ b/students.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -439,6 +439,11 @@
           <t>Age</t>
         </is>
       </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -449,6 +454,11 @@
       <c r="B2" t="n">
         <v>25</v>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Delhi</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -458,6 +468,26 @@
       </c>
       <c r="B3" t="n">
         <v>30</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Mumbai</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Charlie</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>22</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Lucknow</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>